<commit_message>
feat: orion-api routes + performance — blurs eliminados, transiciones 3x mas rapidas
</commit_message>
<xml_diff>
--- a/scripts/output/flota_demo.xlsx
+++ b/scripts/output/flota_demo.xlsx
@@ -451,7 +451,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>4601 VBB</v>
+        <v>8437 KTY</v>
       </c>
       <c r="B2" t="str">
         <v>SEAT</v>
@@ -463,19 +463,19 @@
         <v>TURISMO</v>
       </c>
       <c r="E2" t="str">
-        <v>PARTICULAR</v>
+        <v>SERVICIO PUBLICO</v>
       </c>
       <c r="F2">
         <v>59</v>
       </c>
       <c r="G2">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="H2" t="str">
         <v>NACIONAL</v>
       </c>
       <c r="I2" t="str">
-        <v>TERCEROS AMPLIADO</v>
+        <v>TERCEROS BASICO</v>
       </c>
       <c r="J2" t="str">
         <v>NO</v>
@@ -487,21 +487,21 @@
         <v>SI</v>
       </c>
       <c r="M2">
-        <v>405</v>
+        <v>600</v>
       </c>
       <c r="N2" t="str">
         <v>ALLIANZ</v>
       </c>
       <c r="O2" t="str">
-        <v>AL-2024-008756</v>
+        <v>AL-2024-003976</v>
       </c>
       <c r="P2" t="str">
-        <v>08/09/2026</v>
+        <v>07/08/2026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>1678 YLS</v>
+        <v>9600 KVM</v>
       </c>
       <c r="B3" t="str">
         <v>SEAT</v>
@@ -513,45 +513,45 @@
         <v>TURISMO</v>
       </c>
       <c r="E3" t="str">
-        <v>SERVICIO PUBLICO</v>
+        <v>ALQUILER</v>
       </c>
       <c r="F3">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="G3">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="H3" t="str">
         <v>NACIONAL</v>
       </c>
       <c r="I3" t="str">
-        <v>TERCEROS AMPLIADO</v>
+        <v>TERCEROS BASICO</v>
       </c>
       <c r="J3" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="K3" t="str">
         <v/>
       </c>
       <c r="L3" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
       <c r="M3">
-        <v>636</v>
+        <v>572</v>
       </c>
       <c r="N3" t="str">
         <v>MAPFRE</v>
       </c>
       <c r="O3" t="str">
-        <v>MP-2024-001042</v>
+        <v>MP-2024-007520</v>
       </c>
       <c r="P3" t="str">
-        <v>21/08/2026</v>
+        <v>14/11/2026</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>3445 LNW</v>
+        <v>9102 XRX</v>
       </c>
       <c r="B4" t="str">
         <v>VOLKSWAGEN</v>
@@ -566,42 +566,42 @@
         <v>PARTICULAR</v>
       </c>
       <c r="F4">
-        <v>101</v>
+        <v>128</v>
       </c>
       <c r="G4">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="H4" t="str">
         <v>NACIONAL</v>
       </c>
       <c r="I4" t="str">
-        <v>TODO RIESGO CON FRANQUICIA</v>
+        <v>TODO RIESGO</v>
       </c>
       <c r="J4" t="str">
         <v>NO</v>
       </c>
-      <c r="K4">
-        <v>300</v>
+      <c r="K4" t="str">
+        <v/>
       </c>
       <c r="L4" t="str">
         <v>SI</v>
       </c>
       <c r="M4">
-        <v>677</v>
+        <v>346</v>
       </c>
       <c r="N4" t="str">
         <v>ALLIANZ</v>
       </c>
       <c r="O4" t="str">
-        <v>AL-2024-006602</v>
+        <v>AL-2024-002013</v>
       </c>
       <c r="P4" t="str">
-        <v>01/07/2026</v>
+        <v>22/10/2026</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>4931 SYG</v>
+        <v>7247 BPM</v>
       </c>
       <c r="B5" t="str">
         <v>PEUGEOT</v>
@@ -613,16 +613,16 @@
         <v>TURISMO</v>
       </c>
       <c r="E5" t="str">
-        <v>SERVICIO PUBLICO</v>
+        <v>PARTICULAR</v>
       </c>
       <c r="F5">
-        <v>122</v>
+        <v>83</v>
       </c>
       <c r="G5">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="H5" t="str">
-        <v>NACIONAL</v>
+        <v>PROVINCIAL</v>
       </c>
       <c r="I5" t="str">
         <v>TODO RIESGO CON FRANQUICIA</v>
@@ -631,27 +631,27 @@
         <v>NO</v>
       </c>
       <c r="K5">
-        <v>150</v>
+        <v>600</v>
       </c>
       <c r="L5" t="str">
         <v>SI</v>
       </c>
       <c r="M5">
-        <v>370</v>
+        <v>315</v>
       </c>
       <c r="N5" t="str">
-        <v>AXA</v>
+        <v>MAPFRE</v>
       </c>
       <c r="O5" t="str">
-        <v>AX-2024-005052</v>
+        <v>MP-2024-005307</v>
       </c>
       <c r="P5" t="str">
-        <v>18/10/2026</v>
+        <v>09/07/2026</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>4824 SNK</v>
+        <v>1201 GNV</v>
       </c>
       <c r="B6" t="str">
         <v>BMW</v>
@@ -663,13 +663,13 @@
         <v>TURISMO</v>
       </c>
       <c r="E6" t="str">
-        <v>ALQUILER</v>
+        <v>SERVICIO PUBLICO</v>
       </c>
       <c r="F6">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="G6">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="H6" t="str">
         <v>NACIONAL</v>
@@ -678,30 +678,30 @@
         <v>TERCEROS BASICO</v>
       </c>
       <c r="J6" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="K6" t="str">
         <v/>
       </c>
       <c r="L6" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="M6">
-        <v>752</v>
+        <v>494</v>
       </c>
       <c r="N6" t="str">
         <v>GENERALI</v>
       </c>
       <c r="O6" t="str">
-        <v>GE-2024-006418</v>
+        <v>GE-2024-005852</v>
       </c>
       <c r="P6" t="str">
-        <v>25/08/2026</v>
+        <v>06/09/2026</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>7457 MVY</v>
+        <v>2521 RMK</v>
       </c>
       <c r="B7" t="str">
         <v>RENAULT</v>
@@ -716,10 +716,10 @@
         <v>PARTICULAR</v>
       </c>
       <c r="F7">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G7">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="H7" t="str">
         <v>NACIONAL</v>
@@ -728,30 +728,30 @@
         <v>TODO RIESGO CON FRANQUICIA</v>
       </c>
       <c r="J7" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K7">
+        <v>600</v>
+      </c>
+      <c r="L7" t="str">
         <v>NO</v>
       </c>
-      <c r="K7">
-        <v>300</v>
-      </c>
-      <c r="L7" t="str">
-        <v>SI</v>
-      </c>
       <c r="M7">
-        <v>496</v>
+        <v>670</v>
       </c>
       <c r="N7" t="str">
-        <v>AXA</v>
+        <v>ZURICH</v>
       </c>
       <c r="O7" t="str">
-        <v>AX-2024-006520</v>
+        <v>ZU-2024-005879</v>
       </c>
       <c r="P7" t="str">
-        <v>24/11/2026</v>
+        <v>20/06/2026</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>6593 SMR</v>
+        <v>3457 NNT</v>
       </c>
       <c r="B8" t="str">
         <v>SEAT</v>
@@ -766,42 +766,42 @@
         <v>PARTICULAR</v>
       </c>
       <c r="F8">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="G8">
-        <v>1.6</v>
+        <v>1.5</v>
       </c>
       <c r="H8" t="str">
         <v>NACIONAL</v>
       </c>
       <c r="I8" t="str">
-        <v>TERCEROS BASICO</v>
+        <v>TERCEROS AMPLIADO</v>
       </c>
       <c r="J8" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="K8" t="str">
         <v/>
       </c>
       <c r="L8" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="M8">
-        <v>833</v>
+        <v>764</v>
       </c>
       <c r="N8" t="str">
-        <v>GENERALI</v>
+        <v>ZURICH</v>
       </c>
       <c r="O8" t="str">
-        <v>GE-2024-006631</v>
+        <v>ZU-2024-001488</v>
       </c>
       <c r="P8" t="str">
-        <v>26/12/2026</v>
+        <v>07/09/2026</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>9502 CSY</v>
+        <v>8348 JLJ</v>
       </c>
       <c r="B9" t="str">
         <v>PEUGEOT</v>
@@ -813,7 +813,7 @@
         <v>TODOTERRENO</v>
       </c>
       <c r="E9" t="str">
-        <v>PARTICULAR</v>
+        <v>ALQUILER</v>
       </c>
       <c r="F9">
         <v>118</v>
@@ -825,7 +825,7 @@
         <v>NACIONAL</v>
       </c>
       <c r="I9" t="str">
-        <v>TERCEROS AMPLIADO</v>
+        <v>TODO RIESGO</v>
       </c>
       <c r="J9" t="str">
         <v>SI</v>
@@ -837,21 +837,21 @@
         <v>NO</v>
       </c>
       <c r="M9">
-        <v>300</v>
+        <v>859</v>
       </c>
       <c r="N9" t="str">
-        <v>ZURICH</v>
+        <v>AXA</v>
       </c>
       <c r="O9" t="str">
-        <v>ZU-2024-001457</v>
+        <v>AX-2024-006039</v>
       </c>
       <c r="P9" t="str">
-        <v>08/10/2026</v>
+        <v>19/11/2026</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>6841 KJM</v>
+        <v>7349 NWT</v>
       </c>
       <c r="B10" t="str">
         <v>FORD</v>
@@ -866,42 +866,42 @@
         <v>ALQUILER</v>
       </c>
       <c r="F10">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="G10">
-        <v>3.3</v>
+        <v>3.1</v>
       </c>
       <c r="H10" t="str">
-        <v>NACIONAL</v>
+        <v>PROVINCIAL</v>
       </c>
       <c r="I10" t="str">
-        <v>TODO RIESGO</v>
+        <v>TODO RIESGO CON FRANQUICIA</v>
       </c>
       <c r="J10" t="str">
+        <v>SI</v>
+      </c>
+      <c r="K10">
+        <v>600</v>
+      </c>
+      <c r="L10" t="str">
         <v>NO</v>
       </c>
-      <c r="K10" t="str">
-        <v/>
-      </c>
-      <c r="L10" t="str">
-        <v>SI</v>
-      </c>
       <c r="M10">
-        <v>775</v>
+        <v>736</v>
       </c>
       <c r="N10" t="str">
-        <v>ZURICH</v>
+        <v>GENERALI</v>
       </c>
       <c r="O10" t="str">
-        <v>ZU-2024-005543</v>
+        <v>GE-2024-008911</v>
       </c>
       <c r="P10" t="str">
-        <v>17/07/2026</v>
+        <v>18/09/2026</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>5043 FDH</v>
+        <v>1294 SRP</v>
       </c>
       <c r="B11" t="str">
         <v>MERCEDES-BENZ</v>
@@ -916,10 +916,10 @@
         <v>PARTICULAR</v>
       </c>
       <c r="F11">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G11">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="H11" t="str">
         <v>NACIONAL</v>
@@ -928,30 +928,30 @@
         <v>TERCEROS AMPLIADO</v>
       </c>
       <c r="J11" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="K11" t="str">
         <v/>
       </c>
       <c r="L11" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="M11">
-        <v>653</v>
+        <v>927</v>
       </c>
       <c r="N11" t="str">
-        <v>GENERALI</v>
+        <v>AXA</v>
       </c>
       <c r="O11" t="str">
-        <v>GE-2024-006094</v>
+        <v>AX-2024-009873</v>
       </c>
       <c r="P11" t="str">
-        <v>04/10/2026</v>
+        <v>08/07/2026</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>4276 BKS</v>
+        <v>2062 JBL</v>
       </c>
       <c r="B12" t="str">
         <v>RENAULT</v>
@@ -966,16 +966,16 @@
         <v>PARTICULAR</v>
       </c>
       <c r="F12">
-        <v>105</v>
+        <v>94</v>
       </c>
       <c r="G12">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="H12" t="str">
         <v>NACIONAL</v>
       </c>
       <c r="I12" t="str">
-        <v>TODO RIESGO</v>
+        <v>TERCEROS AMPLIADO</v>
       </c>
       <c r="J12" t="str">
         <v>SI</v>
@@ -984,24 +984,24 @@
         <v/>
       </c>
       <c r="L12" t="str">
-        <v>NO</v>
+        <v>SI</v>
       </c>
       <c r="M12">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="N12" t="str">
         <v>ALLIANZ</v>
       </c>
       <c r="O12" t="str">
-        <v>AL-2024-006509</v>
+        <v>AL-2024-006765</v>
       </c>
       <c r="P12" t="str">
-        <v>04/10/2026</v>
+        <v>07/10/2026</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>7101 YNH</v>
+        <v>6573 FCM</v>
       </c>
       <c r="B13" t="str">
         <v>IVECO</v>
@@ -1013,22 +1013,22 @@
         <v>CAMION</v>
       </c>
       <c r="E13" t="str">
-        <v>ALQUILER</v>
+        <v>PARTICULAR</v>
       </c>
       <c r="F13">
-        <v>149</v>
+        <v>104</v>
       </c>
       <c r="G13">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="H13" t="str">
-        <v>PROVINCIAL</v>
+        <v>NACIONAL</v>
       </c>
       <c r="I13" t="str">
         <v>TERCEROS BASICO</v>
       </c>
       <c r="J13" t="str">
-        <v>SI</v>
+        <v>NO</v>
       </c>
       <c r="K13" t="str">
         <v/>
@@ -1037,16 +1037,16 @@
         <v>SI</v>
       </c>
       <c r="M13">
-        <v>781</v>
+        <v>771</v>
       </c>
       <c r="N13" t="str">
-        <v>GENERALI</v>
+        <v>MAPFRE</v>
       </c>
       <c r="O13" t="str">
-        <v>GE-2024-007678</v>
+        <v>MP-2024-002509</v>
       </c>
       <c r="P13" t="str">
-        <v>09/12/2026</v>
+        <v>23/08/2026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>